<commit_message>
feat: add HU and 3-6 max HRC candidates
</commit_message>
<xml_diff>
--- a/data/stack-sizes/Sizes_for_hrc_script.xlsx
+++ b/data/stack-sizes/Sizes_for_hrc_script.xlsx
@@ -2,7 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R3eae5d4b88a94b22"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3m-6m" sheetId="1" r:id="R0306d7cc67ba416c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HU" sheetId="2" r:id="R87ee85663c854350"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -77,6 +78,27 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">All</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">3.5,7.5</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">3.5,8</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">4,9</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">4,10</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">3bet</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">6,10</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">4bet</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -2088,4 +2110,2008 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" t="s">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="B1">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C1">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="D1">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E1">
+        <x:v>2.5</x:v>
+      </x:c>
+      <x:c r="F1">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G1">
+        <x:v>3.5</x:v>
+      </x:c>
+      <x:c r="H1">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I1">
+        <x:v>4.5</x:v>
+      </x:c>
+      <x:c r="J1">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="K1">
+        <x:v>5.5</x:v>
+      </x:c>
+      <x:c r="L1">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="M1">
+        <x:v>6.5</x:v>
+      </x:c>
+      <x:c r="N1">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="O1">
+        <x:v>7.5</x:v>
+      </x:c>
+      <x:c r="P1">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="Q1">
+        <x:v>8.5</x:v>
+      </x:c>
+      <x:c r="R1">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="S1">
+        <x:v>9.5</x:v>
+      </x:c>
+      <x:c r="T1">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="U1">
+        <x:v>10.5</x:v>
+      </x:c>
+      <x:c r="V1">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="W1">
+        <x:v>11.5</x:v>
+      </x:c>
+      <x:c r="X1">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="Y1">
+        <x:v>12.5</x:v>
+      </x:c>
+      <x:c r="Z1">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="AA1">
+        <x:v>13.5</x:v>
+      </x:c>
+      <x:c r="AB1">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="AC1">
+        <x:v>14.5</x:v>
+      </x:c>
+      <x:c r="AD1">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="AE1">
+        <x:v>15.5</x:v>
+      </x:c>
+      <x:c r="AF1">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="AG1">
+        <x:v>16.5</x:v>
+      </x:c>
+      <x:c r="AH1">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="AI1">
+        <x:v>17.5</x:v>
+      </x:c>
+      <x:c r="AJ1">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="AK1">
+        <x:v>18.5</x:v>
+      </x:c>
+      <x:c r="AL1">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="AM1">
+        <x:v>19.5</x:v>
+      </x:c>
+      <x:c r="AN1">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="AO1">
+        <x:v>20.5</x:v>
+      </x:c>
+      <x:c r="AP1">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="AQ1">
+        <x:v>21.5</x:v>
+      </x:c>
+      <x:c r="AR1">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="AS1">
+        <x:v>22.5</x:v>
+      </x:c>
+      <x:c r="AT1">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="AU1">
+        <x:v>23.5</x:v>
+      </x:c>
+      <x:c r="AV1">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="AW1">
+        <x:v>24.5</x:v>
+      </x:c>
+      <x:c r="AX1">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="AY1">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="AZ1">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="BA1">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="BB1">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="BC1">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="BD1">
+        <x:v>32.5</x:v>
+      </x:c>
+      <x:c r="BE1">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="BF1">
+        <x:v>37.5</x:v>
+      </x:c>
+      <x:c r="BG1">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="BH1">
+        <x:v>42.5</x:v>
+      </x:c>
+      <x:c r="BI1">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="BJ1">
+        <x:v>47.5</x:v>
+      </x:c>
+      <x:c r="BK1">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="BL1">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="BM1">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="BN1">
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="BO1">
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="BP1">
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="BQ1">
+        <x:v>80</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B2" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C2" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D2" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E2" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F2" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G2" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H2" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I2" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="J2" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="K2" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L2" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="M2" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="N2" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="O2" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="P2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="Q2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="R2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="S2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="T2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="U2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="V2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="W2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="X2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="Y2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="Z2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AA2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AB2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AC2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AD2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AE2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AF2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AG2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AH2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AI2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AJ2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AK2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AL2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AM2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AN2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AO2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AP2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AQ2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AR2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AS2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AT2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AU2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AV2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AW2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AX2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AY2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AZ2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="BA2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="BB2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="BC2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="BD2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="BE2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="BF2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="BG2">
+        <x:v>2.25</x:v>
+      </x:c>
+      <x:c r="BH2">
+        <x:v>2.25</x:v>
+      </x:c>
+      <x:c r="BI2">
+        <x:v>2.25</x:v>
+      </x:c>
+      <x:c r="BJ2">
+        <x:v>2.25</x:v>
+      </x:c>
+      <x:c r="BK2">
+        <x:v>2.25</x:v>
+      </x:c>
+      <x:c r="BL2">
+        <x:v>2.25</x:v>
+      </x:c>
+      <x:c r="BM2">
+        <x:v>2.5</x:v>
+      </x:c>
+      <x:c r="BN2">
+        <x:v>2.5</x:v>
+      </x:c>
+      <x:c r="BO2">
+        <x:v>2.5</x:v>
+      </x:c>
+      <x:c r="BP2">
+        <x:v>2.5</x:v>
+      </x:c>
+      <x:c r="BQ2">
+        <x:v>2.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B3" t="str">
+        <x:f>IF(ROUND(B1/15+5/3,2)&gt;=B1*50%,"allin",_xlfn.CONCAT(MIN(ROUND(B1/15+5/3,2),3),IF(MIN(ROUND(0.2*B1+2,2),7)&gt;=B1*50%,"",_xlfn.CONCAT(",",MIN(ROUND(0.2*B1+2,2),7)))))</x:f>
+        <x:v>allin</x:v>
+      </x:c>
+      <x:c r="C3" t="str">
+        <x:f t="shared" ref="C3:BC3" si="0">IF(ROUND(C1/15+5/3,2)&gt;=C1*50%,"allin",_xlfn.CONCAT(MIN(ROUND(C1/15+5/3,2),3),IF(MIN(ROUND(0.2*C1+2,2),7)&gt;=C1*50%,"",_xlfn.CONCAT(",",MIN(ROUND(0.2*C1+2,2),7)))))</x:f>
+        <x:v>allin</x:v>
+      </x:c>
+      <x:c r="D3" t="str">
+        <x:f t="shared" si="0"/>
+        <x:v>allin</x:v>
+      </x:c>
+      <x:c r="E3" t="str">
+        <x:f t="shared" si="0"/>
+        <x:v>allin</x:v>
+      </x:c>
+      <x:c r="F3" t="str">
+        <x:f t="shared" si="0"/>
+        <x:v>allin</x:v>
+      </x:c>
+      <x:c r="G3" t="str">
+        <x:f t="shared" si="0"/>
+        <x:v>allin</x:v>
+      </x:c>
+      <x:c r="H3" t="str">
+        <x:f t="shared" si="0"/>
+        <x:v>1.93</x:v>
+      </x:c>
+      <x:c r="I3" t="str">
+        <x:f t="shared" si="0"/>
+        <x:v>1.97</x:v>
+      </x:c>
+      <x:c r="J3" t="str">
+        <x:f t="shared" si="0"/>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="K3" t="str">
+        <x:f t="shared" si="0"/>
+        <x:v>2.03</x:v>
+      </x:c>
+      <x:c r="L3" t="str">
+        <x:f t="shared" si="0"/>
+        <x:v>2.07</x:v>
+      </x:c>
+      <x:c r="M3" t="str">
+        <x:f t="shared" si="0"/>
+        <x:v>2.1</x:v>
+      </x:c>
+      <x:c r="N3" t="str">
+        <x:f t="shared" si="0"/>
+        <x:v>2.13,3.4</x:v>
+      </x:c>
+      <x:c r="O3" t="str">
+        <x:f t="shared" si="0"/>
+        <x:v>2.17,3.5</x:v>
+      </x:c>
+      <x:c r="P3" t="str">
+        <x:f t="shared" si="0"/>
+        <x:v>2.2,3.6</x:v>
+      </x:c>
+      <x:c r="Q3" t="str">
+        <x:f t="shared" si="0"/>
+        <x:v>2.23,3.7</x:v>
+      </x:c>
+      <x:c r="R3" t="str">
+        <x:f t="shared" si="0"/>
+        <x:v>2.27,3.8</x:v>
+      </x:c>
+      <x:c r="S3" t="str">
+        <x:f t="shared" si="0"/>
+        <x:v>2.3,3.9</x:v>
+      </x:c>
+      <x:c r="T3" t="str">
+        <x:f t="shared" si="0"/>
+        <x:v>2.33,4</x:v>
+      </x:c>
+      <x:c r="U3" t="str">
+        <x:f t="shared" si="0"/>
+        <x:v>2.37,4.1</x:v>
+      </x:c>
+      <x:c r="V3" t="str">
+        <x:f t="shared" si="0"/>
+        <x:v>2.4,4.2</x:v>
+      </x:c>
+      <x:c r="W3" t="str">
+        <x:f t="shared" si="0"/>
+        <x:v>2.43,4.3</x:v>
+      </x:c>
+      <x:c r="X3" t="str">
+        <x:f t="shared" si="0"/>
+        <x:v>2.47,4.4</x:v>
+      </x:c>
+      <x:c r="Y3" t="str">
+        <x:f t="shared" si="0"/>
+        <x:v>2.5,4.5</x:v>
+      </x:c>
+      <x:c r="Z3" t="str">
+        <x:f t="shared" si="0"/>
+        <x:v>2.53,4.6</x:v>
+      </x:c>
+      <x:c r="AA3" t="str">
+        <x:f t="shared" si="0"/>
+        <x:v>2.57,4.7</x:v>
+      </x:c>
+      <x:c r="AB3" t="str">
+        <x:f t="shared" si="0"/>
+        <x:v>2.6,4.8</x:v>
+      </x:c>
+      <x:c r="AC3" t="str">
+        <x:f t="shared" si="0"/>
+        <x:v>2.63,4.9</x:v>
+      </x:c>
+      <x:c r="AD3" t="str">
+        <x:f t="shared" si="0"/>
+        <x:v>2.67,5</x:v>
+      </x:c>
+      <x:c r="AE3" t="str">
+        <x:f t="shared" si="0"/>
+        <x:v>2.7,5.1</x:v>
+      </x:c>
+      <x:c r="AF3" t="str">
+        <x:f t="shared" si="0"/>
+        <x:v>2.73,5.2</x:v>
+      </x:c>
+      <x:c r="AG3" t="str">
+        <x:f t="shared" si="0"/>
+        <x:v>2.77,5.3</x:v>
+      </x:c>
+      <x:c r="AH3" t="str">
+        <x:f t="shared" si="0"/>
+        <x:v>2.8,5.4</x:v>
+      </x:c>
+      <x:c r="AI3" t="str">
+        <x:f t="shared" si="0"/>
+        <x:v>2.83,5.5</x:v>
+      </x:c>
+      <x:c r="AJ3" t="str">
+        <x:f t="shared" si="0"/>
+        <x:v>2.87,5.6</x:v>
+      </x:c>
+      <x:c r="AK3" t="str">
+        <x:f t="shared" si="0"/>
+        <x:v>2.9,5.7</x:v>
+      </x:c>
+      <x:c r="AL3" t="str">
+        <x:f t="shared" si="0"/>
+        <x:v>2.93,5.8</x:v>
+      </x:c>
+      <x:c r="AM3" t="str">
+        <x:f t="shared" si="0"/>
+        <x:v>2.97,5.9</x:v>
+      </x:c>
+      <x:c r="AN3" t="str">
+        <x:f t="shared" si="0"/>
+        <x:v>3,6</x:v>
+      </x:c>
+      <x:c r="AO3" t="str">
+        <x:f t="shared" si="0"/>
+        <x:v>3,6.1</x:v>
+      </x:c>
+      <x:c r="AP3" t="str">
+        <x:f t="shared" si="0"/>
+        <x:v>3,6.2</x:v>
+      </x:c>
+      <x:c r="AQ3" t="str">
+        <x:f t="shared" si="0"/>
+        <x:v>3,6.3</x:v>
+      </x:c>
+      <x:c r="AR3" t="str">
+        <x:f t="shared" si="0"/>
+        <x:v>3,6.4</x:v>
+      </x:c>
+      <x:c r="AS3" t="str">
+        <x:f t="shared" si="0"/>
+        <x:v>3,6.5</x:v>
+      </x:c>
+      <x:c r="AT3" t="str">
+        <x:f t="shared" si="0"/>
+        <x:v>3,6.6</x:v>
+      </x:c>
+      <x:c r="AU3" t="str">
+        <x:f t="shared" si="0"/>
+        <x:v>3,6.7</x:v>
+      </x:c>
+      <x:c r="AV3" t="str">
+        <x:f t="shared" si="0"/>
+        <x:v>3,6.8</x:v>
+      </x:c>
+      <x:c r="AW3" t="str">
+        <x:f t="shared" si="0"/>
+        <x:v>3,6.9</x:v>
+      </x:c>
+      <x:c r="AX3" t="str">
+        <x:f t="shared" si="0"/>
+        <x:v>3,7</x:v>
+      </x:c>
+      <x:c r="AY3" t="str">
+        <x:f t="shared" si="0"/>
+        <x:v>3,7</x:v>
+      </x:c>
+      <x:c r="AZ3" t="str">
+        <x:f t="shared" si="0"/>
+        <x:v>3,7</x:v>
+      </x:c>
+      <x:c r="BA3" t="str">
+        <x:f t="shared" si="0"/>
+        <x:v>3,7</x:v>
+      </x:c>
+      <x:c r="BB3" t="str">
+        <x:f t="shared" si="0"/>
+        <x:v>3,7</x:v>
+      </x:c>
+      <x:c r="BC3" t="str">
+        <x:f t="shared" si="0"/>
+        <x:v>3,7</x:v>
+      </x:c>
+      <x:c r="BD3" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="BE3" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="BF3" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="BG3" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="BH3">
+        <x:v>4.5</x:v>
+      </x:c>
+      <x:c r="BI3">
+        <x:v>4.5</x:v>
+      </x:c>
+      <x:c r="BJ3">
+        <x:v>4.5</x:v>
+      </x:c>
+      <x:c r="BK3">
+        <x:v>4.5</x:v>
+      </x:c>
+      <x:c r="BL3">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="BM3">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="BN3">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="BO3">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="BP3">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="BQ3">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="B5">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C5">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="D5">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E5">
+        <x:v>2.5</x:v>
+      </x:c>
+      <x:c r="F5">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G5">
+        <x:v>3.5</x:v>
+      </x:c>
+      <x:c r="H5">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I5">
+        <x:v>4.5</x:v>
+      </x:c>
+      <x:c r="J5">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="K5">
+        <x:v>5.5</x:v>
+      </x:c>
+      <x:c r="L5">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="M5">
+        <x:v>6.5</x:v>
+      </x:c>
+      <x:c r="N5">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="O5">
+        <x:v>7.5</x:v>
+      </x:c>
+      <x:c r="P5">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="Q5">
+        <x:v>8.5</x:v>
+      </x:c>
+      <x:c r="R5">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="S5">
+        <x:v>9.5</x:v>
+      </x:c>
+      <x:c r="T5">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="U5">
+        <x:v>10.5</x:v>
+      </x:c>
+      <x:c r="V5">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="W5">
+        <x:v>11.5</x:v>
+      </x:c>
+      <x:c r="X5">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="Y5">
+        <x:v>12.5</x:v>
+      </x:c>
+      <x:c r="Z5">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="AA5">
+        <x:v>13.5</x:v>
+      </x:c>
+      <x:c r="AB5">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="AC5">
+        <x:v>14.5</x:v>
+      </x:c>
+      <x:c r="AD5">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="AE5">
+        <x:v>15.5</x:v>
+      </x:c>
+      <x:c r="AF5">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="AG5">
+        <x:v>16.5</x:v>
+      </x:c>
+      <x:c r="AH5">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="AI5">
+        <x:v>17.5</x:v>
+      </x:c>
+      <x:c r="AJ5">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="AK5">
+        <x:v>18.5</x:v>
+      </x:c>
+      <x:c r="AL5">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="AM5">
+        <x:v>19.5</x:v>
+      </x:c>
+      <x:c r="AN5">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="AO5">
+        <x:v>20.5</x:v>
+      </x:c>
+      <x:c r="AP5">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="AQ5">
+        <x:v>21.5</x:v>
+      </x:c>
+      <x:c r="AR5">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="AS5">
+        <x:v>22.5</x:v>
+      </x:c>
+      <x:c r="AT5">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="AU5">
+        <x:v>23.5</x:v>
+      </x:c>
+      <x:c r="AV5">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="AW5">
+        <x:v>24.5</x:v>
+      </x:c>
+      <x:c r="AX5">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="AY5">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="AZ5">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="BA5">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="BB5">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="BC5">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="BD5">
+        <x:v>32.5</x:v>
+      </x:c>
+      <x:c r="BE5">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="BF5">
+        <x:v>37.5</x:v>
+      </x:c>
+      <x:c r="BG5">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="BH5">
+        <x:v>42.5</x:v>
+      </x:c>
+      <x:c r="BI5">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="BJ5">
+        <x:v>47.5</x:v>
+      </x:c>
+      <x:c r="BK5">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="BL5">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="BM5">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="BN5">
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="BO5">
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="BP5">
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="BQ5">
+        <x:v>80</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B6" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C6" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D6" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E6" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F6" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G6" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H6" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I6" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="J6" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="K6" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L6" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="M6" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="N6" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="O6" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="P6" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="Q6" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="R6" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="S6" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="T6" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="U6" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="V6" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="W6" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="X6" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="Y6" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="Z6" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AA6" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AB6" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AC6" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AD6" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AE6" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AF6" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AG6" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AH6" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AI6" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AJ6" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AK6" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AL6" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AM6" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AN6">
+        <x:v>7.5</x:v>
+      </x:c>
+      <x:c r="AO6">
+        <x:v>7.5</x:v>
+      </x:c>
+      <x:c r="AP6">
+        <x:v>7.5</x:v>
+      </x:c>
+      <x:c r="AQ6">
+        <x:v>7.5</x:v>
+      </x:c>
+      <x:c r="AR6">
+        <x:v>7.5</x:v>
+      </x:c>
+      <x:c r="AS6">
+        <x:v>7.5</x:v>
+      </x:c>
+      <x:c r="AT6">
+        <x:v>7.5</x:v>
+      </x:c>
+      <x:c r="AU6">
+        <x:v>7.5</x:v>
+      </x:c>
+      <x:c r="AV6">
+        <x:v>7.5</x:v>
+      </x:c>
+      <x:c r="AW6">
+        <x:v>7.5</x:v>
+      </x:c>
+      <x:c r="AX6">
+        <x:v>7.5</x:v>
+      </x:c>
+      <x:c r="AY6">
+        <x:v>7.5</x:v>
+      </x:c>
+      <x:c r="AZ6">
+        <x:v>7.5</x:v>
+      </x:c>
+      <x:c r="BA6">
+        <x:v>7.5</x:v>
+      </x:c>
+      <x:c r="BB6">
+        <x:v>7.5</x:v>
+      </x:c>
+      <x:c r="BC6">
+        <x:v>7.5</x:v>
+      </x:c>
+      <x:c r="BD6">
+        <x:v>8.5</x:v>
+      </x:c>
+      <x:c r="BE6">
+        <x:v>8.5</x:v>
+      </x:c>
+      <x:c r="BF6">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="BG6">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="BH6">
+        <x:v>10.5</x:v>
+      </x:c>
+      <x:c r="BI6">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="BJ6">
+        <x:v>11.5</x:v>
+      </x:c>
+      <x:c r="BK6">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="BL6">
+        <x:v>12.5</x:v>
+      </x:c>
+      <x:c r="BM6">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="BN6">
+        <x:v>13.5</x:v>
+      </x:c>
+      <x:c r="BO6">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="BP6">
+        <x:v>14.5</x:v>
+      </x:c>
+      <x:c r="BQ6">
+        <x:v>15</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B7" t="str">
+        <x:f>IF(ROUND(B1*0.1+3,2)&gt;=B1*50%,"allin",_xlfn.CONCAT(ROUND(B1*0.1+3,2),IF(MIN(ROUND(B1*0.25+2,2),7)&gt;=B1*50%,"",_xlfn.CONCAT(",",ROUND(B1*0.25+2,2)))))</x:f>
+        <x:v>allin</x:v>
+      </x:c>
+      <x:c r="C7" t="str">
+        <x:f t="shared" ref="C7:BC7" si="1">IF(ROUND(C1*0.1+3,2)&gt;=C1*50%,"allin",_xlfn.CONCAT(ROUND(C1*0.1+3,2),IF(MIN(ROUND(C1*0.25+2,2),7)&gt;=C1*50%,"",_xlfn.CONCAT(",",ROUND(C1*0.25+2,2)))))</x:f>
+        <x:v>allin</x:v>
+      </x:c>
+      <x:c r="D7" t="str">
+        <x:f t="shared" si="1"/>
+        <x:v>allin</x:v>
+      </x:c>
+      <x:c r="E7" t="str">
+        <x:f t="shared" si="1"/>
+        <x:v>allin</x:v>
+      </x:c>
+      <x:c r="F7" t="str">
+        <x:f t="shared" si="1"/>
+        <x:v>allin</x:v>
+      </x:c>
+      <x:c r="G7" t="str">
+        <x:f t="shared" si="1"/>
+        <x:v>allin</x:v>
+      </x:c>
+      <x:c r="H7" t="str">
+        <x:f t="shared" si="1"/>
+        <x:v>allin</x:v>
+      </x:c>
+      <x:c r="I7" t="str">
+        <x:f t="shared" si="1"/>
+        <x:v>allin</x:v>
+      </x:c>
+      <x:c r="J7" t="str">
+        <x:f t="shared" si="1"/>
+        <x:v>allin</x:v>
+      </x:c>
+      <x:c r="K7" t="str">
+        <x:f t="shared" si="1"/>
+        <x:v>allin</x:v>
+      </x:c>
+      <x:c r="L7" t="str">
+        <x:f t="shared" si="1"/>
+        <x:v>allin</x:v>
+      </x:c>
+      <x:c r="M7" t="str">
+        <x:f t="shared" si="1"/>
+        <x:v>allin</x:v>
+      </x:c>
+      <x:c r="N7" t="str">
+        <x:f t="shared" si="1"/>
+        <x:v>allin</x:v>
+      </x:c>
+      <x:c r="O7" t="str">
+        <x:f t="shared" si="1"/>
+        <x:v>allin</x:v>
+      </x:c>
+      <x:c r="P7" t="str">
+        <x:f t="shared" si="1"/>
+        <x:v>3.8</x:v>
+      </x:c>
+      <x:c r="Q7" t="str">
+        <x:f t="shared" si="1"/>
+        <x:v>3.85,4.13</x:v>
+      </x:c>
+      <x:c r="R7" t="str">
+        <x:f t="shared" si="1"/>
+        <x:v>3.9,4.25</x:v>
+      </x:c>
+      <x:c r="S7" t="str">
+        <x:f t="shared" si="1"/>
+        <x:v>3.95,4.38</x:v>
+      </x:c>
+      <x:c r="T7" t="str">
+        <x:f t="shared" si="1"/>
+        <x:v>4,4.5</x:v>
+      </x:c>
+      <x:c r="U7" t="str">
+        <x:f t="shared" si="1"/>
+        <x:v>4.05,4.63</x:v>
+      </x:c>
+      <x:c r="V7" t="str">
+        <x:f t="shared" si="1"/>
+        <x:v>4.1,4.75</x:v>
+      </x:c>
+      <x:c r="W7" t="str">
+        <x:f t="shared" si="1"/>
+        <x:v>4.15,4.88</x:v>
+      </x:c>
+      <x:c r="X7" t="str">
+        <x:f t="shared" si="1"/>
+        <x:v>4.2,5</x:v>
+      </x:c>
+      <x:c r="Y7" t="str">
+        <x:f t="shared" si="1"/>
+        <x:v>4.25,5.13</x:v>
+      </x:c>
+      <x:c r="Z7" t="str">
+        <x:f t="shared" si="1"/>
+        <x:v>4.3,5.25</x:v>
+      </x:c>
+      <x:c r="AA7" t="str">
+        <x:f t="shared" si="1"/>
+        <x:v>4.35,5.38</x:v>
+      </x:c>
+      <x:c r="AB7" t="str">
+        <x:f t="shared" si="1"/>
+        <x:v>4.4,5.5</x:v>
+      </x:c>
+      <x:c r="AC7" t="str">
+        <x:f t="shared" si="1"/>
+        <x:v>4.45,5.63</x:v>
+      </x:c>
+      <x:c r="AD7" t="str">
+        <x:f t="shared" si="1"/>
+        <x:v>4.5,5.75</x:v>
+      </x:c>
+      <x:c r="AE7" t="str">
+        <x:f t="shared" si="1"/>
+        <x:v>4.55,5.88</x:v>
+      </x:c>
+      <x:c r="AF7" t="str">
+        <x:f t="shared" si="1"/>
+        <x:v>4.6,6</x:v>
+      </x:c>
+      <x:c r="AG7" t="str">
+        <x:f t="shared" si="1"/>
+        <x:v>4.65,6.13</x:v>
+      </x:c>
+      <x:c r="AH7" t="str">
+        <x:f t="shared" si="1"/>
+        <x:v>4.7,6.25</x:v>
+      </x:c>
+      <x:c r="AI7" t="str">
+        <x:f t="shared" si="1"/>
+        <x:v>4.75,6.38</x:v>
+      </x:c>
+      <x:c r="AJ7" t="str">
+        <x:f t="shared" si="1"/>
+        <x:v>4.8,6.5</x:v>
+      </x:c>
+      <x:c r="AK7" t="str">
+        <x:f t="shared" si="1"/>
+        <x:v>4.85,6.63</x:v>
+      </x:c>
+      <x:c r="AL7" t="str">
+        <x:f t="shared" si="1"/>
+        <x:v>4.9,6.75</x:v>
+      </x:c>
+      <x:c r="AM7" t="str">
+        <x:f t="shared" si="1"/>
+        <x:v>4.95,6.88</x:v>
+      </x:c>
+      <x:c r="AN7" t="str">
+        <x:f t="shared" si="1"/>
+        <x:v>5,7</x:v>
+      </x:c>
+      <x:c r="AO7" t="str">
+        <x:f t="shared" si="1"/>
+        <x:v>5.05,7.13</x:v>
+      </x:c>
+      <x:c r="AP7" t="str">
+        <x:f t="shared" si="1"/>
+        <x:v>5.1,7.25</x:v>
+      </x:c>
+      <x:c r="AQ7" t="str">
+        <x:f t="shared" si="1"/>
+        <x:v>5.15,7.38</x:v>
+      </x:c>
+      <x:c r="AR7" t="str">
+        <x:f t="shared" si="1"/>
+        <x:v>5.2,7.5</x:v>
+      </x:c>
+      <x:c r="AS7" t="str">
+        <x:f t="shared" si="1"/>
+        <x:v>5.25,7.63</x:v>
+      </x:c>
+      <x:c r="AT7" t="str">
+        <x:f t="shared" si="1"/>
+        <x:v>5.3,7.75</x:v>
+      </x:c>
+      <x:c r="AU7" t="str">
+        <x:f t="shared" si="1"/>
+        <x:v>5.35,7.88</x:v>
+      </x:c>
+      <x:c r="AV7" t="str">
+        <x:f t="shared" si="1"/>
+        <x:v>5.4,8</x:v>
+      </x:c>
+      <x:c r="AW7" t="str">
+        <x:f t="shared" si="1"/>
+        <x:v>5.45,8.13</x:v>
+      </x:c>
+      <x:c r="AX7" t="str">
+        <x:f t="shared" si="1"/>
+        <x:v>5.5,8.25</x:v>
+      </x:c>
+      <x:c r="AY7" t="str">
+        <x:f t="shared" si="1"/>
+        <x:v>5.6,8.5</x:v>
+      </x:c>
+      <x:c r="AZ7" t="str">
+        <x:f t="shared" si="1"/>
+        <x:v>5.7,8.75</x:v>
+      </x:c>
+      <x:c r="BA7" t="str">
+        <x:f t="shared" si="1"/>
+        <x:v>5.8,9</x:v>
+      </x:c>
+      <x:c r="BB7" t="str">
+        <x:f t="shared" si="1"/>
+        <x:v>5.9,9.25</x:v>
+      </x:c>
+      <x:c r="BC7" t="str">
+        <x:f t="shared" si="1"/>
+        <x:v>6,9.5</x:v>
+      </x:c>
+      <x:c r="BD7" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="BE7" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="BF7" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="BG7">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="BH7">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="BI7">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="BJ7">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="BK7">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="BL7">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="BM7">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="BN7">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="BO7">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="BP7">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="BQ7">
+        <x:v>10</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C9">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="D9">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E9">
+        <x:v>2.5</x:v>
+      </x:c>
+      <x:c r="F9">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G9">
+        <x:v>3.5</x:v>
+      </x:c>
+      <x:c r="H9">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I9">
+        <x:v>4.5</x:v>
+      </x:c>
+      <x:c r="J9">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="K9">
+        <x:v>5.5</x:v>
+      </x:c>
+      <x:c r="L9">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="M9">
+        <x:v>6.5</x:v>
+      </x:c>
+      <x:c r="N9">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="O9">
+        <x:v>7.5</x:v>
+      </x:c>
+      <x:c r="P9">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="Q9">
+        <x:v>8.5</x:v>
+      </x:c>
+      <x:c r="R9">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="S9">
+        <x:v>9.5</x:v>
+      </x:c>
+      <x:c r="T9">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="U9">
+        <x:v>10.5</x:v>
+      </x:c>
+      <x:c r="V9">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="W9">
+        <x:v>11.5</x:v>
+      </x:c>
+      <x:c r="X9">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="Y9">
+        <x:v>12.5</x:v>
+      </x:c>
+      <x:c r="Z9">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="AA9">
+        <x:v>13.5</x:v>
+      </x:c>
+      <x:c r="AB9">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="AC9">
+        <x:v>14.5</x:v>
+      </x:c>
+      <x:c r="AD9">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="AE9">
+        <x:v>15.5</x:v>
+      </x:c>
+      <x:c r="AF9">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="AG9">
+        <x:v>16.5</x:v>
+      </x:c>
+      <x:c r="AH9">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="AI9">
+        <x:v>17.5</x:v>
+      </x:c>
+      <x:c r="AJ9">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="AK9">
+        <x:v>18.5</x:v>
+      </x:c>
+      <x:c r="AL9">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="AM9">
+        <x:v>19.5</x:v>
+      </x:c>
+      <x:c r="AN9">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="AO9">
+        <x:v>20.5</x:v>
+      </x:c>
+      <x:c r="AP9">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="AQ9">
+        <x:v>21.5</x:v>
+      </x:c>
+      <x:c r="AR9">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="AS9">
+        <x:v>22.5</x:v>
+      </x:c>
+      <x:c r="AT9">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="AU9">
+        <x:v>23.5</x:v>
+      </x:c>
+      <x:c r="AV9">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="AW9">
+        <x:v>24.5</x:v>
+      </x:c>
+      <x:c r="AX9">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="AY9">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="AZ9">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="BA9">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="BB9">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="BC9">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="BD9">
+        <x:v>32.5</x:v>
+      </x:c>
+      <x:c r="BE9">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="BF9">
+        <x:v>37.5</x:v>
+      </x:c>
+      <x:c r="BG9">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="BH9">
+        <x:v>42.5</x:v>
+      </x:c>
+      <x:c r="BI9">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="BJ9">
+        <x:v>47.5</x:v>
+      </x:c>
+      <x:c r="BK9">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="BL9">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="BM9">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="BN9">
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="BO9">
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="BP9">
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="BQ9">
+        <x:v>80</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B10" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C10" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D10" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E10" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F10" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G10" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H10" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I10" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="J10" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="K10" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L10" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="M10" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="N10" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="O10" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="P10" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="Q10" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="R10" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="S10" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="T10" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="U10" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="V10" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="W10" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="X10" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="Y10" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="Z10" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AA10" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AB10" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AC10" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AD10" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AE10" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AF10" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AG10" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AH10" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AI10" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AJ10" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AK10" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AL10" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AM10" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AN10" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AO10" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AP10" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AQ10" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AR10" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AS10" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AT10" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AU10" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AV10" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AW10" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AX10" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AY10" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AZ10" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="BA10" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="BB10" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="BC10" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="BD10" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="BE10" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="BF10" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="BG10" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="BH10" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="BI10" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="BJ10" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="BK10" t="n">
+        <x:f>BK7*2.25</x:f>
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="BL10" t="n">
+        <x:f t="shared" ref="BL10:BQ10" si="2">BL7*2.25</x:f>
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="BM10">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="BN10">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="BO10">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="BP10">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="BQ10">
+        <x:f t="shared" si="2"/>
+        <x:v>22.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="J11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="K11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="M11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="N11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="O11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="P11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="Q11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="R11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="S11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="T11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="U11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="V11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="W11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="X11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="Y11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="Z11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AA11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AB11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AC11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AD11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AE11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AF11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AG11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AH11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AI11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AJ11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AK11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AL11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AM11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AN11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AO11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AP11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AQ11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AR11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AS11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AT11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AU11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AV11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AW11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AX11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AY11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AZ11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="BA11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="BB11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="BC11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="BD11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="BE11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="BF11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="BG11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="BH11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="BI11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="BJ11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="BK11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="BL11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="BM11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="BN11" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="BO11" t="n">
+        <x:f t="shared" ref="BO11:BP11" si="3">BO6*2</x:f>
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="BP11">
+        <x:f t="shared" si="3"/>
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="BQ11" t="n">
+        <x:f>BQ6*2</x:f>
+        <x:v>30</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>